<commit_message>
更新看板 10月11日 — KPI272.9万(19.4%) 净流水243.8万
</commit_message>
<xml_diff>
--- a/产品分析_导出.xlsx
+++ b/产品分析_导出.xlsx
@@ -463,16 +463,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>390289</v>
+        <v>488348.57</v>
       </c>
       <c r="D2" t="n">
-        <v>1550</v>
+        <v>1955</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>390289</v>
+        <v>488348.57</v>
       </c>
     </row>
     <row r="3">
@@ -487,16 +487,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>334891</v>
+        <v>421051</v>
       </c>
       <c r="D3" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>334891</v>
+        <v>421051</v>
       </c>
     </row>
     <row r="4">
@@ -511,16 +511,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>55398</v>
+        <v>67297.57000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>1484</v>
+        <v>1873</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>55398</v>
+        <v>67297.57000000001</v>
       </c>
     </row>
     <row r="5">
@@ -535,16 +535,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>881376</v>
+        <v>1503890</v>
       </c>
       <c r="D5" t="n">
-        <v>176</v>
+        <v>284</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>881376</v>
+        <v>1503890</v>
       </c>
     </row>
     <row r="6">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>538164</v>
+        <v>974626</v>
       </c>
       <c r="D6" t="n">
-        <v>91</v>
+        <v>155</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>538164</v>
+        <v>974626</v>
       </c>
     </row>
     <row r="7">
@@ -583,16 +583,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>332814</v>
+        <v>498866</v>
       </c>
       <c r="D7" t="n">
-        <v>83</v>
+        <v>126</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>332814</v>
+        <v>498866</v>
       </c>
     </row>
     <row r="8">
@@ -607,16 +607,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>378795.56</v>
+        <v>675688.11</v>
       </c>
       <c r="D8" t="n">
-        <v>432</v>
+        <v>775</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>378795.56</v>
+        <v>675688.11</v>
       </c>
     </row>
     <row r="9">
@@ -627,20 +627,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>复诊</t>
+          <t>初诊</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>198804.33</v>
+        <v>71337.03</v>
       </c>
       <c r="D9" t="n">
-        <v>259</v>
+        <v>86</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>198804.33</v>
+        <v>71337.03</v>
       </c>
     </row>
     <row r="10">
@@ -651,20 +651,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>初诊</t>
+          <t>复诊</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>179991.23</v>
+        <v>55105.91</v>
       </c>
       <c r="D10" t="n">
-        <v>173</v>
+        <v>99</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>179991.23</v>
+        <v>55105.91</v>
       </c>
     </row>
     <row r="11">
@@ -679,16 +679,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>120000</v>
+        <v>144800</v>
       </c>
       <c r="D11" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>120000</v>
+        <v>144800</v>
       </c>
     </row>
     <row r="12">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="13">
@@ -751,16 +751,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1980</v>
+        <v>9900</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>1980</v>
+        <v>9900</v>
       </c>
     </row>
     <row r="15">
@@ -775,16 +775,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8771.360000000001</v>
+        <v>110467.86</v>
       </c>
       <c r="D15" t="n">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>8771.360000000001</v>
+        <v>110467.86</v>
       </c>
     </row>
   </sheetData>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>279698.92</v>
+        <v>570022.17</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -843,11 +843,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>医疗线 279679.92；课程线 19.0</t>
+          <t>医疗线 549245.17；咨询线 20398.0；其他 360.0；课程线 19.0</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>49786</v>
+        <v>62113</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -866,11 +866,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>99.8</v>
+        <v>99.3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>咨询线 49684.0；课程线 102.0</t>
+          <t>咨询线 61674.0；课程线 439.0</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>56438</v>
+        <v>57135</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -889,11 +889,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>68</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>咨询线 38382.0；医疗线 17000.0；其他 999.0；课程线 57.0</t>
+          <t>咨询线 38780.0；医疗线 17000.0；其他 999.0；课程线 356.0</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>120748</v>
+        <v>478417.99</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -912,11 +912,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>52.3</v>
+        <v>72.7</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>咨询线 63198.0；医疗线 37664.0；课程线 17906.0；工作坊 1980.0；其他 0.0</t>
+          <t>咨询线 347576.0；医疗线 56312.99；其他 40000.0；课程线 24629.0；工作坊 9900.0</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>130482.37</v>
+        <v>192656.97</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -935,11 +935,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>89.09999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>咨询线 116292.0；课程线 6657.0；医疗线 6534.37；其他 999.0；菌群线 0.0</t>
+          <t>咨询线 178086.0；医疗线 6914.97；课程线 6657.0；其他 999.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>178784</v>
+        <v>236801</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -958,11 +958,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>74.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>咨询线 133184.0；菌群线 45600.0；课程线 0.0</t>
+          <t>咨询线 184582.0；菌群线 45600.0；课程线 6619.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64413.2</v>
+        <v>87201.2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -981,11 +981,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>86.09999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>咨询线 55476.0；课程线 6619.0；医疗线 2318.2</t>
+          <t>咨询线 78264.0；课程线 6619.0；医疗线 2318.2</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>107777.21</v>
+        <v>166831.25</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1004,11 +1004,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>85</v>
+        <v>77.3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>咨询线 91586.0；考证 10000.0；医疗线 6182.21；课程线 9.0</t>
+          <t>咨询线 128980.0；考证 30000.0；医疗线 7842.25；课程线 9.0</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>45155.1</v>
+        <v>51228.9</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1027,11 +1027,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>96.5</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>咨询线 43594.0；医疗线 1494.1；课程线 67.0</t>
+          <t>咨询线 44788.0；医疗线 6021.4；其他 333.5；课程线 86.0</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15733</v>
+        <v>16952</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1050,11 +1050,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>89</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>咨询线 13996.0；课程线 1737.0；其他 0.0</t>
+          <t>咨询线 15196.0；课程线 1756.0；其他 0.0</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>54407</v>
+        <v>150397</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1073,11 +1073,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>87.8</v>
+        <v>82.3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>咨询线 47788.0；课程线 6619.0</t>
+          <t>咨询线 123778.0；其他 20000.0；课程线 6619.0</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1146,11 +1146,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>李钰坤</t>
+          <t>陈斌斌</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>32180</v>
+        <v>32780</v>
       </c>
     </row>
     <row r="4">
@@ -1164,11 +1164,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>陈斌斌</t>
+          <t>李钰坤</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>27800</v>
+        <v>32180</v>
       </c>
     </row>
     <row r="5">
@@ -1186,7 +1186,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>23620</v>
+        <v>24900</v>
       </c>
     </row>
     <row r="6">
@@ -1200,11 +1200,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>刘士明</t>
+          <t>高曌</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14940</v>
+        <v>21200</v>
       </c>
     </row>
     <row r="7">
@@ -1218,11 +1218,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>陈静</t>
+          <t>岳伟伟</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>70796</v>
+        <v>231208</v>
       </c>
     </row>
     <row r="8">
@@ -1236,11 +1236,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>岳伟伟</t>
+          <t>陈静</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>59616</v>
+        <v>70796</v>
       </c>
     </row>
     <row r="9">
@@ -1254,11 +1254,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>钟燕红</t>
+          <t>陶雯</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>49000</v>
+        <v>62388</v>
       </c>
     </row>
     <row r="10">
@@ -1272,11 +1272,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>张天昂</t>
+          <t>钟燕红</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>43800</v>
+        <v>59398</v>
       </c>
     </row>
     <row r="11">
@@ -1290,11 +1290,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>曾妍妍</t>
+          <t>朱碧丹</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>33394</v>
+        <v>52398</v>
       </c>
     </row>
     <row r="12">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>王倩雅</t>
+          <t>仇晓艳</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>85298.64</v>
+        <v>60977.64</v>
       </c>
     </row>
     <row r="13">
@@ -1326,11 +1326,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>李怡慧</t>
+          <t>仇</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>64963.61</v>
+        <v>39679</v>
       </c>
     </row>
     <row r="14">
@@ -1344,11 +1344,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>韦微</t>
+          <t>小红书</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>50606</v>
+        <v>39316</v>
       </c>
     </row>
     <row r="15">
@@ -1362,11 +1362,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>李菲菲</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>49866</v>
+        <v>32384</v>
       </c>
     </row>
     <row r="16">
@@ -1380,11 +1380,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>李浩然</t>
+          <t>小程序</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29394</v>
+        <v>31691.11</v>
       </c>
     </row>
     <row r="17">
@@ -1452,11 +1452,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>张孟蝶</t>
+          <t>宋晨曦</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>24800</v>
       </c>
     </row>
     <row r="21">
@@ -1488,35 +1488,35 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>陈紫灵</t>
+          <t>林非凡</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>10000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>工作坊</t>
+          <t>考证</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>岳伟伟</t>
+          <t>陈紫灵</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1980</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>工作坊</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1524,17 +1524,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>刘俊彤</t>
+          <t>岳伟伟</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>7920</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>工作坊</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1542,11 +1542,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>岳伟伟</t>
+          <t>陶雯</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="26">
@@ -1556,15 +1556,87 @@
         </is>
       </c>
       <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>陈翔宇</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>高曌</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
         <v>3</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>闫丽东</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>0</v>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>张虹</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>邓璐</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>333.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>5</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>汪贝妮</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -1630,22 +1702,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>390289</v>
+        <v>488348.57</v>
       </c>
       <c r="C2" t="n">
-        <v>67667.03999999999</v>
+        <v>74561.03999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>3611</v>
+        <v>6666</v>
       </c>
       <c r="E2" t="n">
-        <v>0.93</v>
+        <v>1.37</v>
       </c>
       <c r="F2" t="n">
-        <v>64056.04</v>
+        <v>67895.03999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>16.41</v>
+        <v>13.9</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1660,10 +1732,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>881376</v>
+        <v>1503890</v>
       </c>
       <c r="C3" t="n">
-        <v>98600</v>
+        <v>228103.33</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1672,14 +1744,14 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>98600</v>
+        <v>228103.33</v>
       </c>
       <c r="G3" t="n">
-        <v>11.19</v>
+        <v>15.17</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>儿童青少年 65900.0；精神心理 9000.0；暑假礼遇咨询套餐 8500.0</t>
+          <t>儿童青少年 127383.33；家庭守护计划2.0（二阶） 26820.0；电商咨询 26000.0</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1762,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>378795.56</v>
+        <v>675688.11</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -1716,10 +1788,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>120000</v>
+        <v>144800</v>
       </c>
       <c r="C5" t="n">
-        <v>91200</v>
+        <v>92200</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1728,14 +1800,14 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>91200</v>
+        <v>92200</v>
       </c>
       <c r="G5" t="n">
-        <v>76</v>
+        <v>63.67</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>肠道菌群移植（双疗程） 91200.0</t>
+          <t>肠道菌群移植（双疗程） 91200.0；肠道菌群检测（医生专用） 1000.0</t>
         </is>
       </c>
     </row>
@@ -1746,10 +1818,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>27354</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1758,12 +1830,16 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>27354</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
+        <v>91.18000000000001</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>心灯计划-实战派心理咨询师执业培训项目（初阶+中阶） 27354.0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1775,7 +1851,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>87380</v>
+        <v>97180</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -1784,14 +1860,14 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>87380</v>
+        <v>97180</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>青少年成长基地3月营（金盏基地） 46800.0；青少年【未来之翼】身心节律复能7日营 33600.0；蛋壳跳动身心复能营21天（一阶） 5000.0</t>
+          <t>青少年成长基地3月营（金盏基地） 46800.0；青少年【未来之翼】身心节律复能7日营 33600.0；蛋壳跳动身心复能营21天（一阶） 14800.0</t>
         </is>
       </c>
     </row>
@@ -1802,7 +1878,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1980</v>
+        <v>9900</v>
       </c>
       <c r="C8" t="n">
         <v>1980</v>
@@ -1817,7 +1893,7 @@
         <v>1980</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1832,10 +1908,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8771.360000000001</v>
+        <v>110467.86</v>
       </c>
       <c r="C9" t="n">
-        <v>3900</v>
+        <v>4696</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -1844,14 +1920,14 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>3900</v>
+        <v>4696</v>
       </c>
       <c r="G9" t="n">
-        <v>44.46</v>
+        <v>4.25</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>8周系统性心身综合干预+深度服务包（全国统一价） 3900.0</t>
+          <t>8周系统性心身综合干预+深度服务包（全国统一价） 3900.0；门店《一日一生》 796.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
更新看板 10月12日 — KPI333.9万(18.0%) 净流水267.9万
</commit_message>
<xml_diff>
--- a/产品分析_导出.xlsx
+++ b/产品分析_导出.xlsx
@@ -463,16 +463,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>488348.57</v>
+        <v>670171.5699999999</v>
       </c>
       <c r="D2" t="n">
-        <v>1955</v>
+        <v>2264</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>488348.57</v>
+        <v>670171.5699999999</v>
       </c>
     </row>
     <row r="3">
@@ -487,16 +487,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>421051</v>
+        <v>595051</v>
       </c>
       <c r="D3" t="n">
-        <v>82</v>
+        <v>113</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>421051</v>
+        <v>595051</v>
       </c>
     </row>
     <row r="4">
@@ -511,16 +511,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>67297.57000000001</v>
+        <v>75120.57000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>1873</v>
+        <v>2151</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>67297.57000000001</v>
+        <v>75120.57000000001</v>
       </c>
     </row>
     <row r="5">
@@ -535,16 +535,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1503890</v>
+        <v>1582374</v>
       </c>
       <c r="D5" t="n">
-        <v>284</v>
+        <v>307</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>1503890</v>
+        <v>1582374</v>
       </c>
     </row>
     <row r="6">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>974626</v>
+        <v>1019916</v>
       </c>
       <c r="D6" t="n">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>974626</v>
+        <v>1019916</v>
       </c>
     </row>
     <row r="7">
@@ -583,16 +583,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>498866</v>
+        <v>532060</v>
       </c>
       <c r="D7" t="n">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>498866</v>
+        <v>532060</v>
       </c>
     </row>
     <row r="8">
@@ -607,16 +607,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>675688.11</v>
+        <v>684305.78</v>
       </c>
       <c r="D8" t="n">
-        <v>775</v>
+        <v>795</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>675688.11</v>
+        <v>684305.78</v>
       </c>
     </row>
     <row r="9">
@@ -627,20 +627,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>初诊</t>
+          <t>复诊</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>71337.03</v>
+        <v>433234.54</v>
       </c>
       <c r="D9" t="n">
-        <v>86</v>
+        <v>443</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>71337.03</v>
+        <v>433234.54</v>
       </c>
     </row>
     <row r="10">
@@ -651,20 +651,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>复诊</t>
+          <t>初诊</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>55105.91</v>
+        <v>251071.24</v>
       </c>
       <c r="D10" t="n">
-        <v>99</v>
+        <v>352</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>55105.91</v>
+        <v>251071.24</v>
       </c>
     </row>
     <row r="11">
@@ -679,16 +679,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>144800</v>
+        <v>170600</v>
       </c>
       <c r="D11" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>144800</v>
+        <v>170600</v>
       </c>
     </row>
     <row r="12">
@@ -775,16 +775,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>110467.86</v>
+        <v>190467.86</v>
       </c>
       <c r="D15" t="n">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>110467.86</v>
+        <v>190467.86</v>
       </c>
     </row>
   </sheetData>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>570022.17</v>
+        <v>575901.63</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>医疗线 549245.17；咨询线 20398.0；其他 360.0；课程线 19.0</t>
+          <t>医疗线 555124.63；咨询线 20398.0；其他 360.0；课程线 19.0</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>62113</v>
+        <v>69069</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -866,11 +866,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>99.3</v>
+        <v>89.3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>咨询线 61674.0；课程线 439.0</t>
+          <t>咨询线 61674.0；课程线 7395.0</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>478417.99</v>
+        <v>529416.99</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -912,11 +912,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>72.7</v>
+        <v>63.7</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>咨询线 347576.0；医疗线 56312.99；其他 40000.0；课程线 24629.0；工作坊 9900.0</t>
+          <t>咨询线 337176.0；其他 80000.0；医疗线 56612.99；课程线 44728.0；工作坊 9900.0；菌群线 1000.0</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>192656.97</v>
+        <v>203952.18</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -935,11 +935,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>92.40000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>咨询线 178086.0；医疗线 6914.97；课程线 6657.0；其他 999.0；菌群线 0.0</t>
+          <t>咨询线 188882.0；医疗线 7414.18；课程线 6657.0；其他 999.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>236801</v>
+        <v>257597</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -958,11 +958,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>77.90000000000001</v>
+        <v>79.7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>咨询线 184582.0；菌群线 45600.0；课程线 6619.0</t>
+          <t>咨询线 205178.0；菌群线 45600.0；课程线 6619.0；医疗线 200.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>87201.2</v>
+        <v>105001.2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -981,11 +981,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>89.8</v>
+        <v>85.2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>咨询线 78264.0；课程线 6619.0；医疗线 2318.2</t>
+          <t>咨询线 89464.0；课程线 13219.0；医疗线 2318.2；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>166831.25</v>
+        <v>174531.25</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1004,11 +1004,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>77.3</v>
+        <v>78.2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>咨询线 128980.0；考证 30000.0；医疗线 7842.25；课程线 9.0</t>
+          <t>咨询线 136480.0；考证 30000.0；医疗线 8042.25；课程线 9.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>51228.9</v>
+        <v>62024.9</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1027,11 +1027,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>87.40000000000001</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>咨询线 44788.0；医疗线 6021.4；其他 333.5；课程线 86.0</t>
+          <t>咨询线 55584.0；医疗线 6021.4；其他 333.5；课程线 86.0</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16952</v>
+        <v>18651</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1050,11 +1050,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>89.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>咨询线 15196.0；课程线 1756.0；其他 0.0</t>
+          <t>咨询线 15196.0；课程线 3455.0；其他 0.0</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>150397</v>
+        <v>220245</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1073,11 +1073,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>82.3</v>
+        <v>58.5</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>咨询线 123778.0；其他 20000.0；课程线 6619.0</t>
+          <t>咨询线 128778.0；其他 60000.0；菌群线 24800.0；课程线 6667.0</t>
         </is>
       </c>
     </row>
@@ -1128,11 +1128,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>刘孟杰</t>
+          <t>李钰坤</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>34860</v>
+        <v>42140</v>
       </c>
     </row>
     <row r="3">
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>32780</v>
+        <v>37760</v>
       </c>
     </row>
     <row r="4">
@@ -1164,11 +1164,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>李钰坤</t>
+          <t>刘孟杰</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>32180</v>
+        <v>34860</v>
       </c>
     </row>
     <row r="5">
@@ -1182,11 +1182,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>严闽龙</t>
+          <t>高曌</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>24900</v>
+        <v>31160</v>
       </c>
     </row>
     <row r="6">
@@ -1200,11 +1200,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>高曌</t>
+          <t>陶雯</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>21200</v>
+        <v>26400</v>
       </c>
     </row>
     <row r="7">
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>231208</v>
+        <v>220808</v>
       </c>
     </row>
     <row r="8">
@@ -1254,11 +1254,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>陶雯</t>
+          <t>钟燕红</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>62388</v>
+        <v>69796</v>
       </c>
     </row>
     <row r="10">
@@ -1272,11 +1272,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>钟燕红</t>
+          <t>陶雯</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>59398</v>
+        <v>62388</v>
       </c>
     </row>
     <row r="11">
@@ -1290,11 +1290,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>朱碧丹</t>
+          <t>郑巨光</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>52398</v>
+        <v>53194</v>
       </c>
     </row>
     <row r="12">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>仇晓艳</t>
+          <t>王倩雅</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>60977.64</v>
+        <v>128100.6</v>
       </c>
     </row>
     <row r="13">
@@ -1326,11 +1326,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>仇</t>
+          <t>李怡慧</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>39679</v>
+        <v>112331.61</v>
       </c>
     </row>
     <row r="14">
@@ -1344,11 +1344,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>小红书</t>
+          <t>李菲菲</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>39316</v>
+        <v>75946</v>
       </c>
     </row>
     <row r="15">
@@ -1362,11 +1362,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>韦微</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>32384</v>
+        <v>64606</v>
       </c>
     </row>
     <row r="16">
@@ -1380,11 +1380,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>小程序</t>
+          <t>李浩然</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>31691.11</v>
+        <v>63726.2</v>
       </c>
     </row>
     <row r="17">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>王航</t>
+          <t>张虹</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>宋晨曦</t>
+          <t>王航</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1470,11 +1470,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>周玉枝</t>
+          <t>宋晨曦</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>24800</v>
       </c>
     </row>
     <row r="22">
@@ -1560,11 +1560,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>陈翔宇</t>
+          <t>张虹</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="27">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>高曌</t>
+          <t>陈翔宇</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1596,11 +1596,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>张虹</t>
+          <t>高曌</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>20000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="29">
@@ -1614,11 +1614,11 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>邓璐</t>
+          <t>赵越</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>333.5</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="30">
@@ -1632,11 +1632,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>汪贝妮</t>
+          <t>岳伟伟</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>180</v>
+        <v>20000</v>
       </c>
     </row>
   </sheetData>
@@ -1702,26 +1702,26 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>488348.57</v>
+        <v>670171.5699999999</v>
       </c>
       <c r="C2" t="n">
-        <v>74561.03999999999</v>
+        <v>101119.04</v>
       </c>
       <c r="D2" t="n">
-        <v>6666</v>
+        <v>8248</v>
       </c>
       <c r="E2" t="n">
-        <v>1.37</v>
+        <v>1.23</v>
       </c>
       <c r="F2" t="n">
-        <v>67895.03999999999</v>
+        <v>92871.03999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>13.9</v>
+        <v>13.86</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>青少年同行者计划领航营 17542.7；青少年同行者计划护航营（6月） 11685.0；青少年同行者计划-护航营 9826.0</t>
+          <t>青少年同行者计划领航营 42442.7；青少年同行者计划护航营（6月） 11685.0；青少年同行者计划-护航营 9826.0</t>
         </is>
       </c>
     </row>
@@ -1732,10 +1732,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1503890</v>
+        <v>1582374</v>
       </c>
       <c r="C3" t="n">
-        <v>228103.33</v>
+        <v>247521.33</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1744,14 +1744,14 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>228103.33</v>
+        <v>247521.33</v>
       </c>
       <c r="G3" t="n">
-        <v>15.17</v>
+        <v>15.64</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>儿童青少年 127383.33；家庭守护计划2.0（二阶） 26820.0；电商咨询 26000.0</t>
+          <t>儿童青少年 131383.33；家庭守护计划2.0（二阶） 26820.0；电商咨询 26000.0</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>675688.11</v>
+        <v>684305.78</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -1788,7 +1788,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>144800</v>
+        <v>170600</v>
       </c>
       <c r="C5" t="n">
         <v>92200</v>
@@ -1803,7 +1803,7 @@
         <v>92200</v>
       </c>
       <c r="G5" t="n">
-        <v>63.67</v>
+        <v>54.04</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1821,7 +1821,7 @@
         <v>30000</v>
       </c>
       <c r="C6" t="n">
-        <v>27354</v>
+        <v>57080</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1830,14 +1830,14 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>27354</v>
+        <v>57080</v>
       </c>
       <c r="G6" t="n">
-        <v>91.18000000000001</v>
+        <v>190.27</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>心灯计划-实战派心理咨询师执业培训项目（初阶+中阶） 27354.0</t>
+          <t>心灯计划-实战派心理咨询师执业培训项目（初阶+中阶） 57080.0</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>97180</v>
+        <v>150780</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -1860,14 +1860,14 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>97180</v>
+        <v>150780</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>青少年成长基地3月营（金盏基地） 46800.0；青少年【未来之翼】身心节律复能7日营 33600.0；蛋壳跳动身心复能营21天（一阶） 14800.0</t>
+          <t>青少年成长基地3月营（金盏基地） 83600.0；青少年【未来之翼】身心节律复能7日营 33600.0；海南心理能量唤醒营 16800.0</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
         <v>9900</v>
       </c>
       <c r="C8" t="n">
-        <v>1980</v>
+        <v>5940</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -1890,14 +1890,14 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1980</v>
+        <v>5940</v>
       </c>
       <c r="G8" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>【廖文婷】萨提亚家庭系统工作坊 1980.0</t>
+          <t>【廖文婷】萨提亚家庭系统工作坊 5940.0</t>
         </is>
       </c>
     </row>
@@ -1908,10 +1908,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>110467.86</v>
+        <v>190467.86</v>
       </c>
       <c r="C9" t="n">
-        <v>4696</v>
+        <v>5611.75</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -1920,14 +1920,14 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>4696</v>
+        <v>5611.75</v>
       </c>
       <c r="G9" t="n">
-        <v>4.25</v>
+        <v>2.95</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>8周系统性心身综合干预+深度服务包（全国统一价） 3900.0；门店《一日一生》 796.0</t>
+          <t>8周系统性心身综合干预+深度服务包（全国统一价） 3900.0；[自我成长/疗愈] 完形心理认知课，增加智慧。 915.75；门店《一日一生》 796.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
更新看板 10月12日 — KPI333.9万(19.4%) 净流水267.9万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/产品分析_导出.xlsx
+++ b/产品分析_导出.xlsx
@@ -469,10 +469,10 @@
         <v>2264</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>580961.5699999999</v>
       </c>
       <c r="F2" t="n">
-        <v>670171.5699999999</v>
+        <v>89210</v>
       </c>
     </row>
     <row r="3">
@@ -493,10 +493,10 @@
         <v>113</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>509131</v>
       </c>
       <c r="F3" t="n">
-        <v>595051</v>
+        <v>85920</v>
       </c>
     </row>
     <row r="4">
@@ -517,10 +517,10 @@
         <v>2151</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>71830.57000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>75120.57000000001</v>
+        <v>3290</v>
       </c>
     </row>
     <row r="5">
@@ -541,10 +541,10 @@
         <v>307</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>304784</v>
       </c>
       <c r="F5" t="n">
-        <v>1582374</v>
+        <v>1277590</v>
       </c>
     </row>
     <row r="6">
@@ -565,10 +565,10 @@
         <v>170</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>22000</v>
       </c>
       <c r="F6" t="n">
-        <v>1019916</v>
+        <v>997916</v>
       </c>
     </row>
     <row r="7">
@@ -589,10 +589,10 @@
         <v>134</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>282784</v>
       </c>
       <c r="F7" t="n">
-        <v>532060</v>
+        <v>249276</v>
       </c>
     </row>
     <row r="8">
@@ -607,16 +607,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>684305.78</v>
+        <v>685434.5</v>
       </c>
       <c r="D8" t="n">
-        <v>795</v>
+        <v>807</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>31572.13</v>
       </c>
       <c r="F8" t="n">
-        <v>684305.78</v>
+        <v>653862.37</v>
       </c>
     </row>
     <row r="9">
@@ -631,16 +631,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>433234.54</v>
+        <v>434073.26</v>
       </c>
       <c r="D9" t="n">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1107.89</v>
       </c>
       <c r="F9" t="n">
-        <v>433234.54</v>
+        <v>432965.37</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>251071.24</v>
+        <v>251361.24</v>
       </c>
       <c r="D10" t="n">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>30464.24</v>
       </c>
       <c r="F10" t="n">
-        <v>251071.24</v>
+        <v>220897</v>
       </c>
     </row>
     <row r="11">
@@ -685,10 +685,10 @@
         <v>22</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>99200</v>
       </c>
       <c r="F11" t="n">
-        <v>170600</v>
+        <v>71400</v>
       </c>
     </row>
     <row r="12">
@@ -781,10 +781,10 @@
         <v>70</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>47776.36</v>
       </c>
       <c r="F15" t="n">
-        <v>190467.86</v>
+        <v>142691.5</v>
       </c>
     </row>
   </sheetData>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>575901.63</v>
+        <v>596299.63</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -843,11 +843,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>96.40000000000001</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>医疗线 555124.63；咨询线 20398.0；其他 360.0；课程线 19.0</t>
+          <t>医疗线 555124.63；咨询线 40796.0；其他 360.0；课程线 19.0</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>69069</v>
+        <v>48671</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -866,11 +866,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>89.3</v>
+        <v>84.8</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>咨询线 61674.0；课程线 7395.0</t>
+          <t>咨询线 41276.0；课程线 7395.0</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>203952.18</v>
+        <v>205080.9</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -935,11 +935,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>92.59999999999999</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>咨询线 188882.0；医疗线 7414.18；课程线 6657.0；其他 999.0；菌群线 0.0</t>
+          <t>咨询线 188882.0；医疗线 8542.9；课程线 6657.0；其他 999.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>684305.78</v>
+        <v>685434.5</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
更新看板 10月13日 — KPI365.6万(21.3%) 净流水288.7万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/产品分析_导出.xlsx
+++ b/产品分析_导出.xlsx
@@ -463,16 +463,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>670171.5699999999</v>
+        <v>782913.5699999999</v>
       </c>
       <c r="D2" t="n">
-        <v>2264</v>
+        <v>2558</v>
       </c>
       <c r="E2" t="n">
-        <v>580961.5699999999</v>
+        <v>660550.5699999999</v>
       </c>
       <c r="F2" t="n">
-        <v>89210</v>
+        <v>122363</v>
       </c>
     </row>
     <row r="3">
@@ -487,16 +487,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>595051</v>
+        <v>697991</v>
       </c>
       <c r="D3" t="n">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="E3" t="n">
-        <v>509131</v>
+        <v>579071</v>
       </c>
       <c r="F3" t="n">
-        <v>85920</v>
+        <v>118920</v>
       </c>
     </row>
     <row r="4">
@@ -511,16 +511,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>75120.57000000001</v>
+        <v>84922.57000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>2151</v>
+        <v>2431</v>
       </c>
       <c r="E4" t="n">
-        <v>71830.57000000001</v>
+        <v>81479.57000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>3290</v>
+        <v>3443</v>
       </c>
     </row>
     <row r="5">
@@ -535,16 +535,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1582374</v>
+        <v>1750946</v>
       </c>
       <c r="D5" t="n">
-        <v>307</v>
+        <v>352</v>
       </c>
       <c r="E5" t="n">
-        <v>304784</v>
+        <v>316376</v>
       </c>
       <c r="F5" t="n">
-        <v>1277590</v>
+        <v>1434570</v>
       </c>
     </row>
     <row r="6">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1019916</v>
+        <v>1116106</v>
       </c>
       <c r="D6" t="n">
-        <v>170</v>
+        <v>198</v>
       </c>
       <c r="E6" t="n">
-        <v>22000</v>
+        <v>32000</v>
       </c>
       <c r="F6" t="n">
-        <v>997916</v>
+        <v>1084106</v>
       </c>
     </row>
     <row r="7">
@@ -583,16 +583,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>532060</v>
+        <v>596442</v>
       </c>
       <c r="D7" t="n">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="E7" t="n">
-        <v>282784</v>
+        <v>284376</v>
       </c>
       <c r="F7" t="n">
-        <v>249276</v>
+        <v>312066</v>
       </c>
     </row>
     <row r="8">
@@ -607,16 +607,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>685434.5</v>
+        <v>710791.84</v>
       </c>
       <c r="D8" t="n">
-        <v>807</v>
+        <v>896</v>
       </c>
       <c r="E8" t="n">
-        <v>31572.13</v>
+        <v>32427.1</v>
       </c>
       <c r="F8" t="n">
-        <v>653862.37</v>
+        <v>678364.74</v>
       </c>
     </row>
     <row r="9">
@@ -631,16 +631,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>434073.26</v>
+        <v>439387.6</v>
       </c>
       <c r="D9" t="n">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="E9" t="n">
-        <v>1107.89</v>
+        <v>1962.86</v>
       </c>
       <c r="F9" t="n">
-        <v>432965.37</v>
+        <v>437424.74</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>251361.24</v>
+        <v>271404.24</v>
       </c>
       <c r="D10" t="n">
-        <v>358</v>
+        <v>403</v>
       </c>
       <c r="E10" t="n">
         <v>30464.24</v>
       </c>
       <c r="F10" t="n">
-        <v>220897</v>
+        <v>240940</v>
       </c>
     </row>
     <row r="11">
@@ -679,16 +679,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>170600</v>
+        <v>178600</v>
       </c>
       <c r="D11" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E11" t="n">
         <v>99200</v>
       </c>
       <c r="F11" t="n">
-        <v>71400</v>
+        <v>79400</v>
       </c>
     </row>
     <row r="12">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30000</v>
+        <v>30800</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>30000</v>
+        <v>30800</v>
       </c>
     </row>
     <row r="13">
@@ -775,16 +775,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>190467.86</v>
+        <v>192442.86</v>
       </c>
       <c r="D15" t="n">
-        <v>70</v>
+        <v>133</v>
       </c>
       <c r="E15" t="n">
-        <v>47776.36</v>
+        <v>48775.36</v>
       </c>
       <c r="F15" t="n">
-        <v>142691.5</v>
+        <v>143667.5</v>
       </c>
     </row>
   </sheetData>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>596299.63</v>
+        <v>623807.92</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -843,11 +843,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>93.09999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>医疗线 555124.63；咨询线 40796.0；其他 360.0；课程线 19.0</t>
+          <t>医疗线 575852.92；咨询线 40796.0；课程线 6619.0；其他 540.0</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48671</v>
+        <v>81488</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -866,11 +866,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>84.8</v>
+        <v>89.2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>咨询线 41276.0；课程线 7395.0</t>
+          <t>咨询线 72674.0；课程线 7414.0；考证 800.0；医疗线 600.0</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>57135</v>
+        <v>58154</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -889,11 +889,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>67.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>咨询线 38780.0；医疗线 17000.0；其他 999.0；课程线 356.0</t>
+          <t>咨询线 39780.0；医疗线 17000.0；其他 999.0；课程线 375.0</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>529416.99</v>
+        <v>625443.51</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -912,11 +912,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>63.7</v>
+        <v>63.6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>咨询线 337176.0；其他 80000.0；医疗线 56612.99；课程线 44728.0；工作坊 9900.0；菌群线 1000.0</t>
+          <t>咨询线 397772.0；其他 80000.0；课程线 71176.0；医疗线 57595.51；工作坊 9900.0；菌群线 9000.0</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>205080.9</v>
+        <v>227628.9</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>咨询线 188882.0；医疗线 8542.9；课程线 6657.0；其他 999.0；菌群线 0.0</t>
+          <t>咨询线 209680.0；医疗线 10292.9；课程线 6657.0；其他 999.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>257597</v>
+        <v>268393</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -958,11 +958,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>79.7</v>
+        <v>80.3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>咨询线 205178.0；菌群线 45600.0；课程线 6619.0；医疗线 200.0</t>
+          <t>咨询线 215576.0；菌群线 45600.0；课程线 6619.0；其他 398.0；医疗线 200.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>105001.2</v>
+        <v>105466.36</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -985,7 +985,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>咨询线 89464.0；课程线 13219.0；医疗线 2318.2；菌群线 0.0</t>
+          <t>咨询线 89862.0；课程线 13219.0；医疗线 2385.36；其他 0.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>174531.25</v>
+        <v>196472.65</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1004,11 +1004,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>78.2</v>
+        <v>80.3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>咨询线 136480.0；考证 30000.0；医疗线 8042.25；课程线 9.0；菌群线 0.0</t>
+          <t>咨询线 157678.0；考证 30000.0；医疗线 8387.65；其他 398.0；课程线 9.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>62024.9</v>
+        <v>62082.9</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1027,11 +1027,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>89.59999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>咨询线 55584.0；医疗线 6021.4；其他 333.5；课程线 86.0</t>
+          <t>咨询线 55584.0；医疗线 6050.4；其他 333.5；课程线 115.0</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18651</v>
+        <v>19068</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1050,11 +1050,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>81.5</v>
+        <v>81.8</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>咨询线 15196.0；课程线 3455.0；其他 0.0</t>
+          <t>咨询线 15594.0；课程线 3474.0；其他 0.0</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>220245</v>
+        <v>231060</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1073,11 +1073,11 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>58.5</v>
+        <v>60.4</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>咨询线 128778.0；其他 60000.0；菌群线 24800.0；课程线 6667.0</t>
+          <t>咨询线 139574.0；其他 60000.0；菌群线 24800.0；课程线 6686.0</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1128,11 +1128,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>李钰坤</t>
+          <t>刘孟杰</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>42140</v>
+        <v>44820</v>
       </c>
     </row>
     <row r="3">
@@ -1146,11 +1146,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>陈斌斌</t>
+          <t>李钰坤</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>37760</v>
+        <v>42140</v>
       </c>
     </row>
     <row r="4">
@@ -1164,11 +1164,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>刘孟杰</t>
+          <t>陈斌斌</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>34860</v>
+        <v>37760</v>
       </c>
     </row>
     <row r="5">
@@ -1182,11 +1182,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>高曌</t>
+          <t>岳伟伟</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>31160</v>
+        <v>34280</v>
       </c>
     </row>
     <row r="6">
@@ -1200,11 +1200,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>陶雯</t>
+          <t>岳跃峰</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>26400</v>
+        <v>31380</v>
       </c>
     </row>
     <row r="7">
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>220808</v>
+        <v>231604</v>
       </c>
     </row>
     <row r="8">
@@ -1236,11 +1236,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>陈静</t>
+          <t>陶雯</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>70796</v>
+        <v>82188</v>
       </c>
     </row>
     <row r="9">
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>69796</v>
+        <v>80194</v>
       </c>
     </row>
     <row r="10">
@@ -1272,11 +1272,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>陶雯</t>
+          <t>陈静</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>62388</v>
+        <v>70796</v>
       </c>
     </row>
     <row r="11">
@@ -1290,11 +1290,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>郑巨光</t>
+          <t>曾妍妍</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>53194</v>
+        <v>54190</v>
       </c>
     </row>
     <row r="12">
@@ -1330,7 +1330,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>112331.61</v>
+        <v>115986.61</v>
       </c>
     </row>
     <row r="14">
@@ -1344,11 +1344,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>李菲菲</t>
+          <t>李浩然</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>75946</v>
+        <v>84726.2</v>
       </c>
     </row>
     <row r="15">
@@ -1362,11 +1362,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>韦微</t>
+          <t>李菲菲</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>64606</v>
+        <v>77660.28999999999</v>
       </c>
     </row>
     <row r="16">
@@ -1380,11 +1380,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>李浩然</t>
+          <t>余佼</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>63726.2</v>
+        <v>53951</v>
       </c>
     </row>
     <row r="17">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>王航</t>
+          <t>宋晨曦</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>宋晨曦</t>
+          <t>王航</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1516,19 +1516,19 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>工作坊</t>
+          <t>考证</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>岳伟伟</t>
+          <t>褚月月</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>7920</v>
+        <v>800</v>
       </c>
     </row>
     <row r="25">
@@ -1538,33 +1538,33 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>陶雯</t>
+          <t>岳伟伟</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1980</v>
+        <v>7920</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>工作坊</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>张虹</t>
+          <t>陶雯</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>60000</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="27">
@@ -1574,15 +1574,15 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>陈翔宇</t>
+          <t>张虹</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="28">
@@ -1592,11 +1592,11 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>高曌</t>
+          <t>陈翔宇</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1610,15 +1610,15 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>赵越</t>
+          <t>高曌</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>20000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="30">
@@ -1628,14 +1628,32 @@
         </is>
       </c>
       <c r="B30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>岳伟伟</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
         <v>5</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>岳伟伟</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>赵越</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -1702,26 +1720,26 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>670171.5699999999</v>
+        <v>782913.5699999999</v>
       </c>
       <c r="C2" t="n">
-        <v>101119.04</v>
+        <v>132973.04</v>
       </c>
       <c r="D2" t="n">
-        <v>8248</v>
+        <v>8800</v>
       </c>
       <c r="E2" t="n">
-        <v>1.23</v>
+        <v>1.12</v>
       </c>
       <c r="F2" t="n">
-        <v>92871.03999999999</v>
+        <v>124173.04</v>
       </c>
       <c r="G2" t="n">
-        <v>13.86</v>
+        <v>15.86</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>青少年同行者计划领航营 42442.7；青少年同行者计划护航营（6月） 11685.0；青少年同行者计划-护航营 9826.0</t>
+          <t>青少年同行者计划领航营 45759.7；少年说陪伴计划 19800.0；青少年同行者计划 13856.67</t>
         </is>
       </c>
     </row>
@@ -1732,10 +1750,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1582374</v>
+        <v>1750946</v>
       </c>
       <c r="C3" t="n">
-        <v>247521.33</v>
+        <v>279017.33</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1744,14 +1762,14 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>247521.33</v>
+        <v>279017.33</v>
       </c>
       <c r="G3" t="n">
-        <v>15.64</v>
+        <v>15.94</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>儿童青少年 131383.33；家庭守护计划2.0（二阶） 26820.0；电商咨询 26000.0</t>
+          <t>儿童青少年 155781.33；电商咨询 31500.0；家庭守护计划2.0（二阶） 26820.0</t>
         </is>
       </c>
     </row>
@@ -1762,10 +1780,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>685434.5</v>
+        <v>710791.84</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>578</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1774,12 +1792,16 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>578</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
+        <v>0.08</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>20分钟问诊（专家医师） -线上 500.0；AI测评V9.0-多维父母教养行为测评 49.0；AI测评V5.0-原型家庭模式评估 29.0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1788,10 +1810,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>170600</v>
+        <v>178600</v>
       </c>
       <c r="C5" t="n">
-        <v>92200</v>
+        <v>117000</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1800,14 +1822,14 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>92200</v>
+        <v>117000</v>
       </c>
       <c r="G5" t="n">
-        <v>54.04</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>肠道菌群移植（双疗程） 91200.0；肠道菌群检测（医生专用） 1000.0</t>
+          <t>肠道菌群移植（双疗程） 91200.0；肠道菌群移植 24800.0；肠道菌群检测（医生专用） 1000.0</t>
         </is>
       </c>
     </row>
@@ -1818,10 +1840,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30000</v>
+        <v>30800</v>
       </c>
       <c r="C6" t="n">
-        <v>57080</v>
+        <v>76054.88</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1830,14 +1852,14 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>57080</v>
+        <v>76054.88</v>
       </c>
       <c r="G6" t="n">
-        <v>190.27</v>
+        <v>246.93</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>心灯计划-实战派心理咨询师执业培训项目（初阶+中阶） 57080.0</t>
+          <t>心灯计划-实战派心理咨询师执业培训项目（初阶+中阶） 75254.88；[心灯计划]咨询师执业能力培养 (订金，含心理学入门基础实体书) 800.0</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1873,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>150780</v>
+        <v>152280</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -1860,7 +1882,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>150780</v>
+        <v>152280</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1908,10 +1930,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>190467.86</v>
+        <v>192442.86</v>
       </c>
       <c r="C9" t="n">
-        <v>5611.75</v>
+        <v>6009.75</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -1920,14 +1942,14 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>5611.75</v>
+        <v>6009.75</v>
       </c>
       <c r="G9" t="n">
-        <v>2.95</v>
+        <v>3.12</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>8周系统性心身综合干预+深度服务包（全国统一价） 3900.0；[自我成长/疗愈] 完形心理认知课，增加智慧。 915.75；门店《一日一生》 796.0</t>
+          <t>8周系统性心身综合干预+深度服务包（全国统一价） 3900.0；门店《一日一生》 1194.0；[自我成长/疗愈] 完形心理认知课，增加智慧。 915.75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
更新看板 10月14日 — KPI415.5万(24.2%) 净流水328.0万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/产品分析_导出.xlsx
+++ b/产品分析_导出.xlsx
@@ -463,16 +463,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>782913.5699999999</v>
+        <v>922904.5699999999</v>
       </c>
       <c r="D2" t="n">
-        <v>2558</v>
+        <v>2964</v>
       </c>
       <c r="E2" t="n">
-        <v>660550.5699999999</v>
+        <v>766447.5699999999</v>
       </c>
       <c r="F2" t="n">
-        <v>122363</v>
+        <v>156457</v>
       </c>
     </row>
     <row r="3">
@@ -487,16 +487,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>697991</v>
+        <v>825942</v>
       </c>
       <c r="D3" t="n">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="E3" t="n">
-        <v>579071</v>
+        <v>673032</v>
       </c>
       <c r="F3" t="n">
-        <v>118920</v>
+        <v>152910</v>
       </c>
     </row>
     <row r="4">
@@ -511,16 +511,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>84922.57000000001</v>
+        <v>96962.57000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>2431</v>
+        <v>2817</v>
       </c>
       <c r="E4" t="n">
-        <v>81479.57000000001</v>
+        <v>93415.57000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>3443</v>
+        <v>3547</v>
       </c>
     </row>
     <row r="5">
@@ -535,16 +535,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1750946</v>
+        <v>1912854</v>
       </c>
       <c r="D5" t="n">
-        <v>352</v>
+        <v>378</v>
       </c>
       <c r="E5" t="n">
-        <v>316376</v>
+        <v>385594</v>
       </c>
       <c r="F5" t="n">
-        <v>1434570</v>
+        <v>1527260</v>
       </c>
     </row>
     <row r="6">
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1116106</v>
+        <v>1177602</v>
       </c>
       <c r="D6" t="n">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="E6" t="n">
-        <v>32000</v>
+        <v>22000</v>
       </c>
       <c r="F6" t="n">
-        <v>1084106</v>
+        <v>1155602</v>
       </c>
     </row>
     <row r="7">
@@ -583,16 +583,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>596442</v>
+        <v>686854</v>
       </c>
       <c r="D7" t="n">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="E7" t="n">
-        <v>284376</v>
+        <v>363594</v>
       </c>
       <c r="F7" t="n">
-        <v>312066</v>
+        <v>323260</v>
       </c>
     </row>
     <row r="8">
@@ -607,16 +607,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>710791.84</v>
+        <v>835657.71</v>
       </c>
       <c r="D8" t="n">
-        <v>896</v>
+        <v>1032</v>
       </c>
       <c r="E8" t="n">
-        <v>32427.1</v>
+        <v>34268.31</v>
       </c>
       <c r="F8" t="n">
-        <v>678364.74</v>
+        <v>801389.4</v>
       </c>
     </row>
     <row r="9">
@@ -631,16 +631,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>439387.6</v>
+        <v>517802.98</v>
       </c>
       <c r="D9" t="n">
-        <v>493</v>
+        <v>558</v>
       </c>
       <c r="E9" t="n">
-        <v>1962.86</v>
+        <v>2625.58</v>
       </c>
       <c r="F9" t="n">
-        <v>437424.74</v>
+        <v>515177.4</v>
       </c>
     </row>
     <row r="10">
@@ -655,16 +655,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>271404.24</v>
+        <v>317854.73</v>
       </c>
       <c r="D10" t="n">
-        <v>403</v>
+        <v>474</v>
       </c>
       <c r="E10" t="n">
-        <v>30464.24</v>
+        <v>31642.73</v>
       </c>
       <c r="F10" t="n">
-        <v>240940</v>
+        <v>286212</v>
       </c>
     </row>
     <row r="11">
@@ -679,16 +679,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>178600</v>
+        <v>224200</v>
       </c>
       <c r="D11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" t="n">
         <v>99200</v>
       </c>
       <c r="F11" t="n">
-        <v>79400</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="12">
@@ -703,13 +703,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>30800</v>
+        <v>34600</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>3800</v>
       </c>
       <c r="F12" t="n">
         <v>30800</v>
@@ -727,16 +727,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>5940</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>5940</v>
       </c>
     </row>
     <row r="14">
@@ -775,16 +775,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>192442.86</v>
+        <v>209234.86</v>
       </c>
       <c r="D15" t="n">
-        <v>133</v>
+        <v>225</v>
       </c>
       <c r="E15" t="n">
-        <v>48775.36</v>
+        <v>63975.36</v>
       </c>
       <c r="F15" t="n">
-        <v>143667.5</v>
+        <v>145259.5</v>
       </c>
     </row>
   </sheetData>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>623807.92</v>
+        <v>742474.92</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -843,11 +843,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>92.3</v>
+        <v>93.5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>医疗线 575852.92；咨询线 40796.0；课程线 6619.0；其他 540.0</t>
+          <t>医疗线 694500.92；咨询线 40796.0；课程线 6638.0；其他 540.0</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81488</v>
+        <v>83487</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -866,11 +866,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>89.2</v>
+        <v>87</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>咨询线 72674.0；课程线 7414.0；考证 800.0；医疗线 600.0</t>
+          <t>咨询线 72674.0；课程线 7433.0；营地 1980.0；考证 800.0；医疗线 600.0</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>58154</v>
+        <v>79027.84</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -889,11 +889,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>68.40000000000001</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>咨询线 39780.0；医疗线 17000.0；其他 999.0；课程线 375.0</t>
+          <t>咨询线 60178.0；医疗线 17456.84；其他 999.0；课程线 394.0</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>625443.51</v>
+        <v>715177.51</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -912,11 +912,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>63.6</v>
+        <v>57</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>咨询线 397772.0；其他 80000.0；课程线 71176.0；医疗线 57595.51；工作坊 9900.0；菌群线 9000.0</t>
+          <t>咨询线 407772.0；课程线 104214.0；其他 80796.0；医疗线 57895.51；菌群线 54600.0；工作坊 9900.0</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>227628.9</v>
+        <v>231626.72</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -935,11 +935,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>92.09999999999999</v>
+        <v>90.7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>咨询线 209680.0；医疗线 10292.9；课程线 6657.0；其他 999.0；菌群线 0.0</t>
+          <t>咨询线 210078.0；医疗线 13873.72；课程线 6676.0；其他 999.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>268393</v>
+        <v>278412</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -958,11 +958,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>80.3</v>
+        <v>81</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>咨询线 215576.0；菌群线 45600.0；课程线 6619.0；其他 398.0；医疗线 200.0</t>
+          <t>咨询线 225576.0；菌群线 45600.0；课程线 6638.0；其他 398.0；医疗线 200.0</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>105466.36</v>
+        <v>129014.36</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -981,11 +981,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>85.2</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>咨询线 89862.0；课程线 13219.0；医疗线 2385.36；其他 0.0；菌群线 0.0</t>
+          <t>咨询线 108460.0；课程线 14209.0；营地 3960.0；医疗线 2385.36；其他 0.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>196472.65</v>
+        <v>214768.65</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1004,11 +1004,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>80.3</v>
+        <v>81.8</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>咨询线 157678.0；考证 30000.0；医疗线 8387.65；其他 398.0；课程线 9.0；菌群线 0.0</t>
+          <t>咨询线 175576.0；考证 30000.0；医疗线 8387.65；其他 796.0；课程线 9.0；菌群线 0.0</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>62082.9</v>
+        <v>62519.9</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1027,11 +1027,11 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>89.5</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>咨询线 55584.0；医疗线 6050.4；其他 333.5；课程线 115.0</t>
+          <t>咨询线 55584.0；医疗线 6089.4；其他 731.5；课程线 115.0</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19068</v>
+        <v>34466</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1050,11 +1050,11 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>81.8</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>咨询线 15594.0；课程线 3474.0；其他 0.0</t>
+          <t>咨询线 30992.0；课程线 3474.0；其他 0.0</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>231060</v>
+        <v>231031</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>咨询线 139574.0；其他 60000.0；菌群线 24800.0；课程线 6686.0</t>
+          <t>咨询线 139574.0；其他 60000.0；菌群线 24800.0；课程线 6657.0</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1128,11 +1128,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>刘孟杰</t>
+          <t>岳伟伟</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>44820</v>
+        <v>67280</v>
       </c>
     </row>
     <row r="3">
@@ -1146,11 +1146,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>李钰坤</t>
+          <t>岳跃峰</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>42140</v>
+        <v>49560</v>
       </c>
     </row>
     <row r="4">
@@ -1164,11 +1164,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>陈斌斌</t>
+          <t>李钰坤</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>37760</v>
+        <v>47120</v>
       </c>
     </row>
     <row r="5">
@@ -1182,11 +1182,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>岳伟伟</t>
+          <t>刘孟杰</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>34280</v>
+        <v>44820</v>
       </c>
     </row>
     <row r="6">
@@ -1200,11 +1200,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>岳跃峰</t>
+          <t>武存英</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>31380</v>
+        <v>39600</v>
       </c>
     </row>
     <row r="7">
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>82188</v>
+        <v>92188</v>
       </c>
     </row>
     <row r="9">
@@ -1290,11 +1290,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>曾妍妍</t>
+          <t>郑巨光</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>54190</v>
+        <v>63592</v>
       </c>
     </row>
     <row r="12">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>王倩雅</t>
+          <t>李怡慧</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>128100.6</v>
+        <v>167786.61</v>
       </c>
     </row>
     <row r="13">
@@ -1326,11 +1326,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>李怡慧</t>
+          <t>王倩雅</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>115986.61</v>
+        <v>153676.6</v>
       </c>
     </row>
     <row r="14">
@@ -1344,11 +1344,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>李浩然</t>
+          <t>李菲菲</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>84726.2</v>
+        <v>98086.28999999999</v>
       </c>
     </row>
     <row r="15">
@@ -1362,11 +1362,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>李菲菲</t>
+          <t>李浩然</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>77660.28999999999</v>
+        <v>93816.2</v>
       </c>
     </row>
     <row r="16">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>53951</v>
+        <v>60763</v>
       </c>
     </row>
     <row r="17">
@@ -1398,11 +1398,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>武存英</t>
+          <t>岳伟伟</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>49600</v>
+        <v>54600</v>
       </c>
     </row>
     <row r="18">
@@ -1416,11 +1416,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>李颜君</t>
+          <t>武存英</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>45600</v>
+        <v>49600</v>
       </c>
     </row>
     <row r="19">
@@ -1434,11 +1434,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>张虹</t>
+          <t>李颜君</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>24800</v>
+        <v>45600</v>
       </c>
     </row>
     <row r="20">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>宋晨曦</t>
+          <t>张虹</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1524,101 +1524,101 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>褚月月</t>
+          <t>陈斌斌</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>800</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>工作坊</t>
+          <t>考证</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>岳伟伟</t>
+          <t>褚月月</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>7920</v>
+        <v>800</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>工作坊</t>
+          <t>营地</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>陶雯</t>
+          <t>冯兰兰</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1980</v>
+        <v>3960</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>营地</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>张虹</t>
+          <t>刘馨</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>60000</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>工作坊</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>陈翔宇</t>
+          <t>岳伟伟</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>40000</v>
+        <v>7920</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>工作坊</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>高曌</t>
+          <t>陶雯</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>40000</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="30">
@@ -1628,15 +1628,15 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>岳伟伟</t>
+          <t>张虹</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>20000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="31">
@@ -1646,14 +1646,68 @@
         </is>
       </c>
       <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>陈翔宇</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>高曌</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>岳伟伟</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>20796</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
         <v>5</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>赵越</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D34" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -1720,26 +1774,26 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>782913.5699999999</v>
+        <v>922904.5699999999</v>
       </c>
       <c r="C2" t="n">
-        <v>132973.04</v>
+        <v>156150.74</v>
       </c>
       <c r="D2" t="n">
-        <v>8800</v>
+        <v>9511</v>
       </c>
       <c r="E2" t="n">
-        <v>1.12</v>
+        <v>1.03</v>
       </c>
       <c r="F2" t="n">
-        <v>124173.04</v>
+        <v>146639.74</v>
       </c>
       <c r="G2" t="n">
-        <v>15.86</v>
+        <v>15.89</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>青少年同行者计划领航营 45759.7；少年说陪伴计划 19800.0；青少年同行者计划 13856.67</t>
+          <t>青少年同行者计划领航营 50739.7；少年说陪伴计划 26400.0；青少年同行者计划向阳营 14593.37</t>
         </is>
       </c>
     </row>
@@ -1750,10 +1804,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1750946</v>
+        <v>1912854</v>
       </c>
       <c r="C3" t="n">
-        <v>279017.33</v>
+        <v>315517.33</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1762,14 +1816,14 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>279017.33</v>
+        <v>315517.33</v>
       </c>
       <c r="G3" t="n">
-        <v>15.94</v>
+        <v>16.49</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>儿童青少年 155781.33；电商咨询 31500.0；家庭守护计划2.0（二阶） 26820.0</t>
+          <t>儿童青少年 181781.33；精神心理 31696.0；电商咨询 31500.0</t>
         </is>
       </c>
     </row>
@@ -1780,26 +1834,26 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>710791.84</v>
+        <v>835657.71</v>
       </c>
       <c r="C4" t="n">
-        <v>578</v>
+        <v>3178</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>578</v>
+        <v>2578</v>
       </c>
       <c r="G4" t="n">
-        <v>0.08</v>
+        <v>0.31</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>20分钟问诊（专家医师） -线上 500.0；AI测评V9.0-多维父母教养行为测评 49.0；AI测评V5.0-原型家庭模式评估 29.0</t>
+          <t>线上/线下门诊 1800.0；20分钟问诊（医师） -线上 800.0；20分钟问诊（专家医师） -线上 500.0</t>
         </is>
       </c>
     </row>
@@ -1810,10 +1864,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>178600</v>
+        <v>224200</v>
       </c>
       <c r="C5" t="n">
-        <v>117000</v>
+        <v>138800</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1822,14 +1876,14 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>117000</v>
+        <v>138800</v>
       </c>
       <c r="G5" t="n">
-        <v>65.51000000000001</v>
+        <v>61.91</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>肠道菌群移植（双疗程） 91200.0；肠道菌群移植 24800.0；肠道菌群检测（医生专用） 1000.0</t>
+          <t>肠道菌群移植（双疗程） 91200.0；肠道菌群移植 24800.0；肠道菌群移植（双疗程优惠） 20800.0</t>
         </is>
       </c>
     </row>
@@ -1840,10 +1894,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30800</v>
+        <v>34600</v>
       </c>
       <c r="C6" t="n">
-        <v>76054.88</v>
+        <v>77633.17999999999</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1852,14 +1906,14 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>76054.88</v>
+        <v>77633.17999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>246.93</v>
+        <v>224.37</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>心灯计划-实战派心理咨询师执业培训项目（初阶+中阶） 75254.88；[心灯计划]咨询师执业能力培养 (订金，含心理学入门基础实体书) 800.0</t>
+          <t>心灯计划-实战派心理咨询师执业培训项目（初阶+中阶） 75254.88；心理咨询取证班+实操案例直播课+群内答疑+讲义=3188 1578.3；[心灯计划]咨询师执业能力培养 (订金，含心理学入门基础实体书) 800.0</t>
         </is>
       </c>
     </row>
@@ -1870,10 +1924,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>5940</v>
       </c>
       <c r="C7" t="n">
-        <v>152280</v>
+        <v>172080</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -1882,14 +1936,14 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>152280</v>
+        <v>172080</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>2896.97</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>青少年成长基地3月营（金盏基地） 83600.0；青少年【未来之翼】身心节律复能7日营 33600.0；海南心理能量唤醒营 16800.0</t>
+          <t>青少年成长基地3月营（金盏基地） 83600.0；蛋壳跳动身心复能营21天（一阶） 34600.0；青少年【未来之翼】身心节律复能7日营 33600.0</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1984,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>192442.86</v>
+        <v>209234.86</v>
       </c>
       <c r="C9" t="n">
         <v>6009.75</v>
@@ -1945,7 +1999,7 @@
         <v>6009.75</v>
       </c>
       <c r="G9" t="n">
-        <v>3.12</v>
+        <v>2.87</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>

</xml_diff>